<commit_message>
Update S-curve template: Vazirmatn font, right-to-left cells
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJ3LJCBkip2JqmScgxTPHH
</commit_message>
<xml_diff>
--- a/free/axislabs-s-curve.xlsx
+++ b/free/axislabs-s-curve.xlsx
@@ -375,12 +375,11 @@
     <numFmt numFmtId="171" formatCode="General"/>
     <numFmt numFmtId="172" formatCode="0%;[RED]\-0%;0%"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <name val="Vazirmatn"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -402,14 +401,14 @@
       <b val="true"/>
       <sz val="15"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF94A3B8"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -417,42 +416,42 @@
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF475569"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF475569"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="12"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF008000"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -460,13 +459,7 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Tahoma"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -474,7 +467,7 @@
       <i val="true"/>
       <sz val="8"/>
       <color rgb="FF94A3B8"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -519,7 +512,7 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF2563EB"/>
-      <name val="Tahoma"/>
+      <name val="Vazirmatn"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -611,55 +604,55 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -667,71 +660,71 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="2"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -746,7 +739,7 @@
   <dxfs count="5">
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="Vazirmatn"/>
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
@@ -760,7 +753,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="Vazirmatn"/>
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
@@ -774,7 +767,7 @@
     </dxf>
     <dxf>
       <font>
-        <name val="Tahoma"/>
+        <name val="Vazirmatn"/>
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
@@ -888,7 +881,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>منحنی S — برنامه‌ای در برابر واقعی</a:t>
+              <a:t>منحنی پیشرفت: برنامه‌ای در برابر واقعی</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1329,11 +1322,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="91267607"/>
-        <c:axId val="98787429"/>
+        <c:axId val="76800876"/>
+        <c:axId val="39612064"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="91267607"/>
+        <c:axId val="76800876"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1399,7 +1392,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98787429"/>
+        <c:crossAx val="39612064"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1407,7 +1400,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98787429"/>
+        <c:axId val="39612064"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -1475,7 +1468,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91267607"/>
+        <c:crossAx val="76800876"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1532,15 +1525,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>-61920</xdr:colOff>
+      <xdr:colOff>-180360</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>39600</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>169920</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1548,7 +1541,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-14578200" y="762120"/>
+        <a:off x="-13386960" y="762120"/>
         <a:ext cx="7199640" cy="3959640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1743,10 +1736,10 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:J43"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
@@ -1781,7 +1774,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1795,7 +1788,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
@@ -1803,7 +1796,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
@@ -1811,7 +1804,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
@@ -1819,7 +1812,7 @@
         <v>46102</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
         <v>7</v>
       </c>
@@ -1832,7 +1825,7 @@
         <v>0.466666666666667</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="E9" s="9" t="s">
@@ -1843,7 +1836,7 @@
         <v>0.375</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
       <c r="E10" s="9" t="s">
@@ -1854,7 +1847,7 @@
         <v>-0.0916666666666667</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
       <c r="E11" s="9" t="s">
@@ -1865,7 +1858,7 @@
         <v>0.803571428571429</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
       <c r="E12" s="9" t="s">
@@ -1876,7 +1869,7 @@
         <v>عقب‌افتاده</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="4" t="s">
         <v>13</v>
       </c>
@@ -1906,7 +1899,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="n">
         <v>1</v>
       </c>
@@ -1931,7 +1924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="n">
         <v>2</v>
       </c>
@@ -1956,7 +1949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="n">
         <v>3</v>
       </c>
@@ -1981,7 +1974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="n">
         <v>4</v>
       </c>
@@ -2006,7 +1999,7 @@
         <v>0.977358490566038</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="n">
         <v>5</v>
       </c>
@@ -2031,7 +2024,7 @@
         <v>0.942452830188679</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="n">
         <v>6</v>
       </c>
@@ -2056,7 +2049,7 @@
         <v>0.9288</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="n">
         <v>7</v>
       </c>
@@ -2081,7 +2074,7 @@
         <v>0.916804979253112</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="n">
         <v>8</v>
       </c>
@@ -2106,7 +2099,7 @@
         <v>0.850089445438283</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="n">
         <v>9</v>
       </c>
@@ -2131,7 +2124,7 @@
         <v>0.85188679245283</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="n">
         <v>10</v>
       </c>
@@ -2156,7 +2149,7 @@
         <v>0.821739130434783</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="n">
         <v>11</v>
       </c>
@@ -2181,7 +2174,7 @@
         <v>0.825949367088608</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="n">
         <v>12</v>
       </c>
@@ -2206,7 +2199,7 @@
         <v>0.803571428571429</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="n">
         <v>13</v>
       </c>
@@ -2231,7 +2224,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="n">
         <v>14</v>
       </c>
@@ -2256,7 +2249,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="n">
         <v>15</v>
       </c>
@@ -2281,7 +2274,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="n">
         <v>16</v>
       </c>
@@ -2306,7 +2299,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="n">
         <v>17</v>
       </c>
@@ -2331,7 +2324,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16" t="n">
         <v>18</v>
       </c>
@@ -2356,7 +2349,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="n">
         <v>19</v>
       </c>
@@ -2381,7 +2374,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="n">
         <v>20</v>
       </c>
@@ -2406,7 +2399,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="n">
         <v>21</v>
       </c>
@@ -2431,7 +2424,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="16" t="n">
         <v>22</v>
       </c>
@@ -2456,7 +2449,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="n">
         <v>23</v>
       </c>
@@ -2481,7 +2474,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="n">
         <v>24</v>
       </c>
@@ -2506,7 +2499,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="n">
         <v>25</v>
       </c>
@@ -2531,7 +2524,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="n">
         <v>26</v>
       </c>
@@ -2614,7 +2607,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="95"/>
@@ -2723,7 +2716,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -2759,7 +2752,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>38</v>
       </c>
@@ -2801,7 +2794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>47</v>
       </c>
@@ -2834,7 +2827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
         <v>49</v>
       </c>
@@ -2867,7 +2860,7 @@
         <v>-0.05</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
         <v>51</v>
       </c>
@@ -2900,7 +2893,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>53</v>
       </c>
@@ -2933,7 +2926,7 @@
         <v>-0.1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>55</v>
       </c>
@@ -2966,7 +2959,7 @@
         <v>-0.216666666666667</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>57</v>
       </c>
@@ -2999,7 +2992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>59</v>
       </c>
@@ -3032,7 +3025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
         <v>61</v>
       </c>
@@ -3226,7 +3219,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="27" t="s">
         <v>63</v>
       </c>
@@ -3270,10 +3263,11 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="3" style="0" width="8.5"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3426,7 +3420,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A6="","",'فعالیت‌ها'!A6)</f>
         <v>A1</v>
@@ -3540,7 +3534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A7="","",'فعالیت‌ها'!A7)</f>
         <v>A2</v>
@@ -3654,7 +3648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A8="","",'فعالیت‌ها'!A8)</f>
         <v>A3</v>
@@ -3768,7 +3762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A9="","",'فعالیت‌ها'!A9)</f>
         <v>A4</v>
@@ -3882,7 +3876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A10="","",'فعالیت‌ها'!A10)</f>
         <v>A5</v>
@@ -3996,7 +3990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A11="","",'فعالیت‌ها'!A11)</f>
         <v>A6</v>
@@ -4110,7 +4104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A12="","",'فعالیت‌ها'!A12)</f>
         <v>A7</v>
@@ -4224,7 +4218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A13="","",'فعالیت‌ها'!A13)</f>
         <v>A8</v>
@@ -4338,7 +4332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A14="","",'فعالیت‌ها'!A14)</f>
         <v/>
@@ -4452,7 +4446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A15="","",'فعالیت‌ها'!A15)</f>
         <v/>
@@ -4566,7 +4560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A16="","",'فعالیت‌ها'!A16)</f>
         <v/>
@@ -4680,7 +4674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A17="","",'فعالیت‌ها'!A17)</f>
         <v/>
@@ -4794,7 +4788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A18="","",'فعالیت‌ها'!A18)</f>
         <v/>
@@ -4908,7 +4902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A19="","",'فعالیت‌ها'!A19)</f>
         <v/>
@@ -5022,7 +5016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A20="","",'فعالیت‌ها'!A20)</f>
         <v/>
@@ -5157,10 +5151,11 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AB20"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="3" style="0" width="8.5"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5313,7 +5308,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A6="","",'فعالیت‌ها'!A6)</f>
         <v>A1</v>
@@ -5373,7 +5368,7 @@
       <c r="AA6" s="24"/>
       <c r="AB6" s="24"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A7="","",'فعالیت‌ها'!A7)</f>
         <v>A2</v>
@@ -5431,7 +5426,7 @@
       <c r="AA7" s="24"/>
       <c r="AB7" s="24"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A8="","",'فعالیت‌ها'!A8)</f>
         <v>A3</v>
@@ -5485,7 +5480,7 @@
       <c r="AA8" s="24"/>
       <c r="AB8" s="24"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A9="","",'فعالیت‌ها'!A9)</f>
         <v>A4</v>
@@ -5537,7 +5532,7 @@
       <c r="AA9" s="24"/>
       <c r="AB9" s="24"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A10="","",'فعالیت‌ها'!A10)</f>
         <v>A5</v>
@@ -5585,7 +5580,7 @@
       <c r="AA10" s="24"/>
       <c r="AB10" s="24"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A11="","",'فعالیت‌ها'!A11)</f>
         <v>A6</v>
@@ -5621,7 +5616,7 @@
       <c r="AA11" s="24"/>
       <c r="AB11" s="24"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A12="","",'فعالیت‌ها'!A12)</f>
         <v>A7</v>
@@ -5657,7 +5652,7 @@
       <c r="AA12" s="24"/>
       <c r="AB12" s="24"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="str">
         <f aca="false">IF('فعالیت‌ها'!A13="","",'فعالیت‌ها'!A13)</f>
         <v>A8</v>

</xml_diff>